<commit_message>
03052026 - testmanifeste analyse IV
</commit_message>
<xml_diff>
--- a/tabelle der testmanifeste.xlsx
+++ b/tabelle der testmanifeste.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="141">
   <si>
     <t>Name</t>
   </si>
@@ -490,6 +490,17 @@
   </si>
   <si>
     <t>Offen!</t>
+  </si>
+  <si>
+    <t>Wenn ich ehrlich bin, läuft bei mir eigentlich immer irgendwas. Musik ist kein Bewusstseinszustand bei mir, sie ist einfach da. Der Kern ist elektronisch – Techno, Acid, Drum &amp; Bass, Minimal – und das ist keine Phase, das ist Haltung. Eine kreischende 303 über einem fetten Bass mit einer Melodie die sich irgendwo dazwischenschiebt: mehr brauche ich nicht um einen Abend als gelungen zu betrachten. Dass ich auch mit Sting oder Led Zeppelin oder NIN was anfangen kann, erwähne ich nur der Vollständigkeit halber. Das Herzstück ist und bleibt das Elektronische. Ich drehe selbst gelegentlich an Reglern – nichts für die Öffentlichkeit, aber der Prozess macht mir was. Wenn die Muse da ist. Manchmal ist sie das.
+Ich hab mir meinen Lebensort bewusst ausgesucht. Lützow ist kein Kompromiss, das ist Absicht. Vorher Rostock, und der Grund für beides ist derselbe: Wasser. Meer. Diese Möglichkeit, einfach raus zu gehen und auf etwas zu schauen, das größer ist als der eigene Kopf. Gleichzeitig pendle ich nach Frankfurt wenn die Arbeit es verlangt – IT, also meistens remote, manchmal nicht. Dieser Wechsel zwischen Großstadt und dem kleinen Ort hier ist für mich kein notwendiges Übel, das ist ein aktiv genutzter Kontrast. Hamburg liegt auf der Strecke und ich mag Hamburg, das sei noch gesagt.
+Unterwegs bin ich gern – zu Fuß, mit dem Rad, nachts durch eine Stadt ohne bestimmtes Ziel. Am Strand sitzen und aufs Meer starren ohne dabei irgendetwas leisten zu müssen ist für mich keine verschwendete Zeit. Das ist eigentlich die direkteste Form von Erholung, die ich kenne.
+Ich fotografiere wenn die Zeit es zulässt. Menschen, Straßen, Momente die sich ergeben. Kein Studio, kein Setup.
+Politisch bin ich links verortet. Das ist keine große Ansage, das ist einfach wie ich die Welt lese. Ob ich drüber reden will hängt von der Person und dem Moment ab – ich find das Thema wichtig, aber ich muss nicht bei jedem Abend damit anfangen.
+Alkohol ist bei mir so gut wie kein Thema. Rauchen leider schon – kein Tabak, IQOS, was ich selbst nicht als Verbesserung verkaufen würde, nur als weniger aggressiv für die Umgebung. Ich weiß es, ich hab's akzeptiert, vorerst.</t>
+  </si>
+  <si>
+    <t>marcankertest</t>
   </si>
 </sst>
 </file>
@@ -907,7 +918,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:M70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
@@ -1041,12 +1052,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="120" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="285" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>12</v>
@@ -1055,136 +1066,136 @@
         <v>18</v>
       </c>
       <c r="E4" s="5">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F4" s="5">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I4" s="5">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>53</v>
+        <v>103</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>54</v>
+        <v>139</v>
       </c>
       <c r="M4" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="105" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E5" s="5">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="F5" s="5">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I5" s="5">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="M5" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="105" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E6" s="5">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F6" s="5">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I6" s="5">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M6" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="120" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E7" s="5">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="F7" s="5">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>66</v>
+        <v>17</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>16</v>
@@ -1193,36 +1204,36 @@
         <v>150</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="M7" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="105" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>108</v>
+        <v>65</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>108</v>
+        <v>65</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E8" s="5">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="F8" s="5">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>66</v>
@@ -1231,139 +1242,139 @@
         <v>16</v>
       </c>
       <c r="I8" s="5">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>109</v>
+        <v>67</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>106</v>
+        <v>68</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>110</v>
+        <v>64</v>
       </c>
       <c r="M8" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="90" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>61</v>
+        <v>108</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>61</v>
+        <v>108</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E9" s="5">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F9" s="5">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I9" s="5">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>63</v>
+        <v>106</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="M9" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="90" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>114</v>
+        <v>61</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>114</v>
+        <v>61</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E10" s="5">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="F10" s="5">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I10" s="5">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>116</v>
+        <v>63</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M10" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E11" s="5">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F11" s="5">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I11" s="5">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>115</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="M11" s="12">
         <v>1</v>
@@ -1371,107 +1382,107 @@
     </row>
     <row r="12" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E12" s="5">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="F12" s="5">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I12" s="5">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="M12" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="105" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C13" s="8" t="s">
+    <row r="13" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E13" s="7">
-        <v>43</v>
-      </c>
-      <c r="F13" s="7">
-        <v>149</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I13" s="7">
-        <v>250</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="K13" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="L13" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="M13" s="7" t="s">
-        <v>86</v>
+      <c r="D13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" s="5">
+        <v>49</v>
+      </c>
+      <c r="F13" s="5">
+        <v>167</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" s="5">
+        <v>200</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="M13" s="12">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E14" s="7">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="F14" s="7">
-        <v>162</v>
+        <v>149</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>16</v>
@@ -1480,13 +1491,13 @@
         <v>250</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M14" s="7" t="s">
         <v>86</v>
@@ -1494,40 +1505,40 @@
     </row>
     <row r="15" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E15" s="7">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="F15" s="7">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I15" s="7">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="M15" s="7" t="s">
         <v>86</v>
@@ -1535,22 +1546,22 @@
     </row>
     <row r="16" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E16" s="7">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F16" s="7">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>17</v>
@@ -1562,13 +1573,13 @@
         <v>200</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>81</v>
+        <v>47</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="M16" s="7" t="s">
         <v>86</v>
@@ -1576,25 +1587,25 @@
     </row>
     <row r="17" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E17" s="7">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F17" s="7">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>16</v>
@@ -1603,95 +1614,95 @@
         <v>200</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="M17" s="7" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="105" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E18" s="7">
+        <v>35</v>
+      </c>
+      <c r="F18" s="7">
+        <v>159</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" s="7">
+        <v>200</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="105" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B19" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C19" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E18" s="9">
+      <c r="D19" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" s="9">
         <v>45</v>
       </c>
-      <c r="F18" s="9">
+      <c r="F19" s="9">
         <v>165</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G19" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="H18" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="I18" s="9">
+      <c r="H19" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" s="9">
         <v>200</v>
       </c>
-      <c r="J18" s="9" t="s">
+      <c r="J19" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="K18" s="9" t="s">
+      <c r="K19" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="L18" s="9" t="s">
+      <c r="L19" s="9" t="s">
         <v>90</v>
-      </c>
-      <c r="M18" s="9" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="90" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E19" s="9">
-        <v>39</v>
-      </c>
-      <c r="F19" s="9">
-        <v>164</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="H19" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="I19" s="9">
-        <v>250</v>
-      </c>
-      <c r="J19" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="K19" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="L19" s="9" t="s">
-        <v>94</v>
       </c>
       <c r="M19" s="9" t="s">
         <v>91</v>
@@ -1699,66 +1710,66 @@
     </row>
     <row r="20" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>18</v>
       </c>
       <c r="E20" s="9">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="F20" s="9">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I20" s="9">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>20</v>
+        <v>93</v>
       </c>
       <c r="L20" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M20" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="90" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>18</v>
       </c>
       <c r="E21" s="9">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="F21" s="9">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="H21" s="9" t="s">
         <v>16</v>
@@ -1767,13 +1778,13 @@
         <v>200</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="M21" s="9" t="s">
         <v>91</v>
@@ -1781,66 +1792,66 @@
     </row>
     <row r="22" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>18</v>
       </c>
       <c r="E22" s="9">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="F22" s="9">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>105</v>
+        <v>17</v>
       </c>
       <c r="H22" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I22" s="9">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>62</v>
+        <v>102</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="M22" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="150" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>12</v>
+        <v>104</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>13</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>18</v>
       </c>
       <c r="E23" s="9">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F23" s="9">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="H23" s="9" t="s">
         <v>16</v>
@@ -1849,121 +1860,121 @@
         <v>250</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>124</v>
+        <v>62</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="M23" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="165" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" ht="150" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>128</v>
+        <v>123</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>123</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>18</v>
       </c>
       <c r="E24" s="9">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F24" s="9">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I24" s="9">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="L24" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M24" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="150" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" ht="165" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>18</v>
       </c>
       <c r="E25" s="9">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F25" s="9">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="H25" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I25" s="9">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>30</v>
+        <v>129</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>20</v>
+        <v>130</v>
       </c>
       <c r="L25" s="9" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="M25" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="180" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" ht="150" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D26" s="9" t="s">
         <v>18</v>
       </c>
       <c r="E26" s="9">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="F26" s="9">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="H26" s="9" t="s">
         <v>16</v>
@@ -1972,159 +1983,159 @@
         <v>250</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>135</v>
+        <v>20</v>
       </c>
       <c r="L26" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="M26" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="165" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" ht="180" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>70</v>
+        <v>134</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>70</v>
+        <v>134</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>18</v>
       </c>
       <c r="E27" s="9">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F27" s="9">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="H27" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I27" s="9">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>88</v>
+        <v>62</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="L27" s="9" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="M27" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="90" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C28" s="16" t="s">
+    <row r="28" spans="1:13" ht="165" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D28" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="E28" s="15">
-        <v>48</v>
-      </c>
-      <c r="F28" s="15">
-        <v>185</v>
-      </c>
-      <c r="G28" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="H28" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="I28" s="15">
-        <v>200</v>
-      </c>
-      <c r="J28" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K28" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="M28" s="17" t="s">
-        <v>138</v>
+      <c r="D28" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E28" s="9">
+        <v>45</v>
+      </c>
+      <c r="F28" s="9">
+        <v>168</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" s="9">
+        <v>100</v>
+      </c>
+      <c r="J28" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="K28" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="L28" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="M28" s="9" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E29" s="15">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F29" s="15">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="G29" s="15" t="s">
         <v>17</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I29" s="15">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J29" s="15" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="K29" s="15" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="M29" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E30" s="15">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="F30" s="15">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="G30" s="15" t="s">
         <v>17</v>
@@ -2133,39 +2144,39 @@
         <v>16</v>
       </c>
       <c r="I30" s="15">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="J30" s="15" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="K30" s="15" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="M30" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="315" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E31" s="15">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="F31" s="15">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G31" s="15" t="s">
         <v>17</v>
@@ -2174,39 +2185,39 @@
         <v>16</v>
       </c>
       <c r="I31" s="15">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="J31" s="15" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="K31" s="15" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="M31" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="165" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" ht="315" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D32" s="15" t="s">
         <v>18</v>
       </c>
       <c r="E32" s="15">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F32" s="15">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="G32" s="15" t="s">
         <v>17</v>
@@ -2215,64 +2226,102 @@
         <v>16</v>
       </c>
       <c r="I32" s="15">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="J32" s="15" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="K32" s="15" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M32" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="180" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" ht="165" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E33" s="15">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="F33" s="15">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="G33" s="15" t="s">
         <v>17</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I33" s="15">
         <v>100</v>
       </c>
       <c r="J33" s="15" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="K33" s="15" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="M33" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="L34" s="1"/>
+    <row r="34" spans="1:13" ht="180" x14ac:dyDescent="0.25">
+      <c r="A34" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="E34" s="15">
+        <v>41</v>
+      </c>
+      <c r="F34" s="15">
+        <v>181</v>
+      </c>
+      <c r="G34" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H34" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="I34" s="15">
+        <v>100</v>
+      </c>
+      <c r="J34" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="K34" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="M34" s="17" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L35" s="1"/>
@@ -2379,42 +2428,46 @@
     <row r="69" spans="12:12" x14ac:dyDescent="0.25">
       <c r="L69" s="1"/>
     </row>
+    <row r="70" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L70" s="1"/>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C28" r:id="rId1"/>
-    <hyperlink ref="C29" r:id="rId2"/>
-    <hyperlink ref="C30" r:id="rId3"/>
-    <hyperlink ref="C31" r:id="rId4"/>
-    <hyperlink ref="C32" r:id="rId5"/>
-    <hyperlink ref="C33" r:id="rId6"/>
+    <hyperlink ref="C29" r:id="rId1"/>
+    <hyperlink ref="C30" r:id="rId2"/>
+    <hyperlink ref="C31" r:id="rId3"/>
+    <hyperlink ref="C32" r:id="rId4"/>
+    <hyperlink ref="C33" r:id="rId5"/>
+    <hyperlink ref="C34" r:id="rId6"/>
     <hyperlink ref="C2" r:id="rId7"/>
     <hyperlink ref="C3" r:id="rId8"/>
-    <hyperlink ref="C4" r:id="rId9"/>
-    <hyperlink ref="C5" r:id="rId10"/>
-    <hyperlink ref="C6" r:id="rId11"/>
-    <hyperlink ref="C7" r:id="rId12"/>
-    <hyperlink ref="C13" r:id="rId13"/>
-    <hyperlink ref="C14" r:id="rId14"/>
-    <hyperlink ref="C15" r:id="rId15"/>
-    <hyperlink ref="C16" r:id="rId16"/>
-    <hyperlink ref="C17" r:id="rId17"/>
-    <hyperlink ref="C18" r:id="rId18"/>
-    <hyperlink ref="C19" r:id="rId19"/>
-    <hyperlink ref="C20" r:id="rId20"/>
-    <hyperlink ref="C21" r:id="rId21"/>
-    <hyperlink ref="C22" r:id="rId22"/>
-    <hyperlink ref="C8" r:id="rId23"/>
-    <hyperlink ref="C9" r:id="rId24"/>
-    <hyperlink ref="C10" r:id="rId25"/>
-    <hyperlink ref="C11" r:id="rId26"/>
-    <hyperlink ref="C12" r:id="rId27"/>
-    <hyperlink ref="C23" r:id="rId28"/>
-    <hyperlink ref="C24" r:id="rId29"/>
-    <hyperlink ref="C25" r:id="rId30"/>
-    <hyperlink ref="C26" r:id="rId31"/>
-    <hyperlink ref="C27" r:id="rId32"/>
+    <hyperlink ref="C5" r:id="rId9"/>
+    <hyperlink ref="C6" r:id="rId10"/>
+    <hyperlink ref="C7" r:id="rId11"/>
+    <hyperlink ref="C8" r:id="rId12"/>
+    <hyperlink ref="C14" r:id="rId13"/>
+    <hyperlink ref="C15" r:id="rId14"/>
+    <hyperlink ref="C16" r:id="rId15"/>
+    <hyperlink ref="C17" r:id="rId16"/>
+    <hyperlink ref="C18" r:id="rId17"/>
+    <hyperlink ref="C19" r:id="rId18"/>
+    <hyperlink ref="C20" r:id="rId19"/>
+    <hyperlink ref="C21" r:id="rId20"/>
+    <hyperlink ref="C22" r:id="rId21"/>
+    <hyperlink ref="C23" r:id="rId22"/>
+    <hyperlink ref="C9" r:id="rId23"/>
+    <hyperlink ref="C10" r:id="rId24"/>
+    <hyperlink ref="C11" r:id="rId25"/>
+    <hyperlink ref="C12" r:id="rId26"/>
+    <hyperlink ref="C13" r:id="rId27"/>
+    <hyperlink ref="C24" r:id="rId28"/>
+    <hyperlink ref="C25" r:id="rId29"/>
+    <hyperlink ref="C26" r:id="rId30"/>
+    <hyperlink ref="C27" r:id="rId31"/>
+    <hyperlink ref="C28" r:id="rId32"/>
+    <hyperlink ref="C4" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId33"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId34"/>
 </worksheet>
 </file>
</xml_diff>